<commit_message>
bacukp 22 de febrero
</commit_message>
<xml_diff>
--- a/data/registro_actual.xlsx
+++ b/data/registro_actual.xlsx
@@ -7,14 +7,14 @@
     <workbookView xWindow="240" yWindow="15" windowWidth="16095" windowHeight="9660"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="Registro" sheetId="1" r:id="rId1"/>
   </sheets>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="45" uniqueCount="43">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="64" uniqueCount="54">
   <si>
     <t>Nombre_Facultad</t>
   </si>
@@ -100,24 +100,45 @@
     <t>Facultad_de_Ciencias_de_la_Salud</t>
   </si>
   <si>
+    <t>Facultad_de_Ciencias_Jurídicas</t>
+  </si>
+  <si>
     <t>Especialización en Medicina Crítica y Cuidados Intensivos</t>
   </si>
   <si>
+    <t>Derecho</t>
+  </si>
+  <si>
     <t>Elvia Lucía Sanchez García</t>
   </si>
   <si>
+    <t>Carlos Morales</t>
+  </si>
+  <si>
     <t>Juan Pablo Charry</t>
   </si>
   <si>
+    <t>María Eugenia Nieto</t>
+  </si>
+  <si>
     <t>Temas_Centro_Escritura</t>
   </si>
   <si>
+    <t>APA _(7 ed. 2020)_American_Psychological_Association.</t>
+  </si>
+  <si>
     <t>Alfonso, Virtual</t>
   </si>
   <si>
+    <t>Gonzalo Gallego, Presencial</t>
+  </si>
+  <si>
     <t>Cien años de soledad</t>
   </si>
   <si>
+    <t>Prueba</t>
+  </si>
+  <si>
     <t>Álvaro Agudelo</t>
   </si>
   <si>
@@ -130,16 +151,28 @@
     <t>Sí</t>
   </si>
   <si>
+    <t>No</t>
+  </si>
+  <si>
     <t>Presencial</t>
   </si>
   <si>
+    <t>Virtual</t>
+  </si>
+  <si>
     <t>Temas_Centro_Escritura | IEEE_(2025)_Institute_of_Electrical_and_Electronics_Engineers</t>
   </si>
   <si>
     <t>Juan Pablo Charry | Diego López, Presencial | Diego Alejandro Soto</t>
   </si>
   <si>
+    <t>2026-02-23</t>
+  </si>
+  <si>
     <t>EN PROCESO</t>
+  </si>
+  <si>
+    <t>Si</t>
   </si>
   <si>
     <t>alfonso</t>
@@ -504,7 +537,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AA2"/>
+  <dimension ref="A1:AA3"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:27">
@@ -595,67 +628,138 @@
         <v>27</v>
       </c>
       <c r="B2" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="C2">
         <v>1053766068</v>
       </c>
       <c r="D2" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="E2" t="s">
-        <v>30</v>
+        <v>33</v>
       </c>
       <c r="F2" t="s">
-        <v>31</v>
+        <v>35</v>
       </c>
       <c r="H2" t="s">
-        <v>32</v>
+        <v>37</v>
       </c>
       <c r="I2" t="s">
-        <v>33</v>
+        <v>39</v>
       </c>
       <c r="J2" s="2">
         <v>46073</v>
       </c>
       <c r="K2" t="s">
-        <v>34</v>
+        <v>41</v>
       </c>
       <c r="L2" t="s">
-        <v>35</v>
+        <v>42</v>
       </c>
       <c r="N2" t="s">
-        <v>36</v>
+        <v>43</v>
       </c>
       <c r="P2" t="s">
-        <v>37</v>
+        <v>44</v>
       </c>
       <c r="Q2">
         <v>0</v>
       </c>
       <c r="R2" t="s">
-        <v>37</v>
+        <v>44</v>
       </c>
       <c r="S2" t="s">
-        <v>38</v>
+        <v>46</v>
       </c>
       <c r="T2">
         <v>2</v>
       </c>
       <c r="U2" t="s">
-        <v>39</v>
+        <v>48</v>
       </c>
       <c r="V2" t="s">
+        <v>49</v>
+      </c>
+      <c r="X2" t="s">
+        <v>51</v>
+      </c>
+      <c r="Z2" t="s">
+        <v>33</v>
+      </c>
+      <c r="AA2" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="3" spans="1:27">
+      <c r="A3" t="s">
+        <v>28</v>
+      </c>
+      <c r="B3" t="s">
+        <v>30</v>
+      </c>
+      <c r="C3">
+        <v>123456</v>
+      </c>
+      <c r="D3" t="s">
+        <v>32</v>
+      </c>
+      <c r="E3" t="s">
+        <v>34</v>
+      </c>
+      <c r="F3" t="s">
+        <v>36</v>
+      </c>
+      <c r="H3" t="s">
+        <v>38</v>
+      </c>
+      <c r="I3" t="s">
         <v>40</v>
       </c>
-      <c r="X2" t="s">
+      <c r="J3" s="2">
+        <v>46076</v>
+      </c>
+      <c r="K3" t="s">
         <v>41</v>
       </c>
-      <c r="Z2" t="s">
-        <v>30</v>
-      </c>
-      <c r="AA2" t="s">
+      <c r="L3" t="s">
         <v>42</v>
+      </c>
+      <c r="M3" t="s">
+        <v>43</v>
+      </c>
+      <c r="N3" t="s">
+        <v>43</v>
+      </c>
+      <c r="P3" t="s">
+        <v>44</v>
+      </c>
+      <c r="Q3">
+        <v>4</v>
+      </c>
+      <c r="R3" t="s">
+        <v>45</v>
+      </c>
+      <c r="S3" t="s">
+        <v>47</v>
+      </c>
+      <c r="T3">
+        <v>1</v>
+      </c>
+      <c r="U3" t="s">
+        <v>36</v>
+      </c>
+      <c r="W3" t="s">
+        <v>50</v>
+      </c>
+      <c r="X3" t="s">
+        <v>52</v>
+      </c>
+      <c r="Z3" t="s">
+        <v>34</v>
+      </c>
+      <c r="AA3" t="s">
+        <v>38</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
cambio de storage de almacenamiento
</commit_message>
<xml_diff>
--- a/data/registro_actual.xlsx
+++ b/data/registro_actual.xlsx
@@ -7,14 +7,14 @@
     <workbookView xWindow="240" yWindow="15" windowWidth="16095" windowHeight="9660"/>
   </bookViews>
   <sheets>
-    <sheet name="Registro" sheetId="1" r:id="rId1"/>
+    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="64" uniqueCount="54">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="80" uniqueCount="60">
   <si>
     <t>Nombre_Facultad</t>
   </si>
@@ -103,24 +103,39 @@
     <t>Facultad_de_Ciencias_Jurídicas</t>
   </si>
   <si>
+    <t>Facultad_de_Ciencias_Contables_Económicas_y_Administrativas</t>
+  </si>
+  <si>
     <t>Especialización en Medicina Crítica y Cuidados Intensivos</t>
   </si>
   <si>
     <t>Derecho</t>
   </si>
   <si>
+    <t>Administración de Empresas</t>
+  </si>
+  <si>
+    <t>1053805543</t>
+  </si>
+  <si>
     <t>Elvia Lucía Sanchez García</t>
   </si>
   <si>
     <t>Carlos Morales</t>
   </si>
   <si>
+    <t>sebas</t>
+  </si>
+  <si>
     <t>Juan Pablo Charry</t>
   </si>
   <si>
     <t>María Eugenia Nieto</t>
   </si>
   <si>
+    <t>Harold Estiven García</t>
+  </si>
+  <si>
     <t>Temas_Centro_Escritura</t>
   </si>
   <si>
@@ -142,9 +157,6 @@
     <t>Álvaro Agudelo</t>
   </si>
   <si>
-    <t>Harold Estiven García</t>
-  </si>
-  <si>
     <t>ok</t>
   </si>
   <si>
@@ -169,10 +181,16 @@
     <t>2026-02-23</t>
   </si>
   <si>
+    <t>2026-02-22</t>
+  </si>
+  <si>
     <t>EN PROCESO</t>
   </si>
   <si>
     <t>Si</t>
+  </si>
+  <si>
+    <t>En proceso</t>
   </si>
   <si>
     <t>alfonso</t>
@@ -537,7 +555,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AA3"/>
+  <dimension ref="A1:AA4"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:27">
@@ -628,67 +646,67 @@
         <v>27</v>
       </c>
       <c r="B2" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="C2">
         <v>1053766068</v>
       </c>
       <c r="D2" t="s">
-        <v>31</v>
+        <v>34</v>
       </c>
       <c r="E2" t="s">
-        <v>33</v>
+        <v>37</v>
       </c>
       <c r="F2" t="s">
-        <v>35</v>
+        <v>40</v>
       </c>
       <c r="H2" t="s">
-        <v>37</v>
+        <v>42</v>
       </c>
       <c r="I2" t="s">
-        <v>39</v>
+        <v>44</v>
       </c>
       <c r="J2" s="2">
         <v>46073</v>
       </c>
       <c r="K2" t="s">
-        <v>41</v>
+        <v>46</v>
       </c>
       <c r="L2" t="s">
-        <v>42</v>
+        <v>39</v>
       </c>
       <c r="N2" t="s">
-        <v>43</v>
+        <v>47</v>
       </c>
       <c r="P2" t="s">
-        <v>44</v>
+        <v>48</v>
       </c>
       <c r="Q2">
         <v>0</v>
       </c>
       <c r="R2" t="s">
-        <v>44</v>
+        <v>48</v>
       </c>
       <c r="S2" t="s">
-        <v>46</v>
+        <v>50</v>
       </c>
       <c r="T2">
         <v>2</v>
       </c>
       <c r="U2" t="s">
-        <v>48</v>
+        <v>52</v>
       </c>
       <c r="V2" t="s">
-        <v>49</v>
+        <v>53</v>
       </c>
       <c r="X2" t="s">
-        <v>51</v>
+        <v>56</v>
       </c>
       <c r="Z2" t="s">
-        <v>33</v>
+        <v>37</v>
       </c>
       <c r="AA2" t="s">
-        <v>53</v>
+        <v>59</v>
       </c>
     </row>
     <row r="3" spans="1:27">
@@ -696,70 +714,129 @@
         <v>28</v>
       </c>
       <c r="B3" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="C3">
         <v>123456</v>
       </c>
       <c r="D3" t="s">
-        <v>32</v>
+        <v>35</v>
       </c>
       <c r="E3" t="s">
-        <v>34</v>
+        <v>38</v>
       </c>
       <c r="F3" t="s">
-        <v>36</v>
+        <v>41</v>
       </c>
       <c r="H3" t="s">
-        <v>38</v>
+        <v>43</v>
       </c>
       <c r="I3" t="s">
-        <v>40</v>
+        <v>45</v>
       </c>
       <c r="J3" s="2">
         <v>46076</v>
       </c>
       <c r="K3" t="s">
-        <v>41</v>
+        <v>46</v>
       </c>
       <c r="L3" t="s">
-        <v>42</v>
+        <v>39</v>
       </c>
       <c r="M3" t="s">
-        <v>43</v>
+        <v>47</v>
       </c>
       <c r="N3" t="s">
-        <v>43</v>
+        <v>47</v>
       </c>
       <c r="P3" t="s">
-        <v>44</v>
+        <v>48</v>
       </c>
       <c r="Q3">
         <v>4</v>
       </c>
       <c r="R3" t="s">
-        <v>45</v>
+        <v>49</v>
       </c>
       <c r="S3" t="s">
-        <v>47</v>
+        <v>51</v>
       </c>
       <c r="T3">
         <v>1</v>
       </c>
       <c r="U3" t="s">
+        <v>41</v>
+      </c>
+      <c r="W3" t="s">
+        <v>54</v>
+      </c>
+      <c r="X3" t="s">
+        <v>57</v>
+      </c>
+      <c r="Z3" t="s">
+        <v>38</v>
+      </c>
+      <c r="AA3" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="4" spans="1:27">
+      <c r="A4" t="s">
+        <v>29</v>
+      </c>
+      <c r="B4" t="s">
+        <v>32</v>
+      </c>
+      <c r="C4" t="s">
+        <v>33</v>
+      </c>
+      <c r="D4" t="s">
         <v>36</v>
       </c>
-      <c r="W3" t="s">
-        <v>50</v>
-      </c>
-      <c r="X3" t="s">
-        <v>52</v>
-      </c>
-      <c r="Z3" t="s">
-        <v>34</v>
-      </c>
-      <c r="AA3" t="s">
-        <v>38</v>
+      <c r="E4" t="s">
+        <v>39</v>
+      </c>
+      <c r="F4" t="s">
+        <v>41</v>
+      </c>
+      <c r="I4" t="s">
+        <v>44</v>
+      </c>
+      <c r="J4" s="2">
+        <v>46075</v>
+      </c>
+      <c r="K4" t="s">
+        <v>46</v>
+      </c>
+      <c r="L4" t="s">
+        <v>39</v>
+      </c>
+      <c r="P4" t="s">
+        <v>48</v>
+      </c>
+      <c r="Q4">
+        <v>0</v>
+      </c>
+      <c r="R4" t="s">
+        <v>48</v>
+      </c>
+      <c r="S4" t="s">
+        <v>51</v>
+      </c>
+      <c r="T4">
+        <v>1</v>
+      </c>
+      <c r="U4" t="s">
+        <v>41</v>
+      </c>
+      <c r="W4" t="s">
+        <v>55</v>
+      </c>
+      <c r="X4" t="s">
+        <v>58</v>
+      </c>
+      <c r="Z4" t="s">
+        <v>39</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
restablecimiento de appy con almacenamiento en excel
</commit_message>
<xml_diff>
--- a/data/registro_actual.xlsx
+++ b/data/registro_actual.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="80" uniqueCount="60">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="45" uniqueCount="43">
   <si>
     <t>Nombre_Facultad</t>
   </si>
@@ -100,97 +100,46 @@
     <t>Facultad_de_Ciencias_de_la_Salud</t>
   </si>
   <si>
-    <t>Facultad_de_Ciencias_Jurídicas</t>
-  </si>
-  <si>
-    <t>Facultad_de_Ciencias_Contables_Económicas_y_Administrativas</t>
-  </si>
-  <si>
     <t>Especialización en Medicina Crítica y Cuidados Intensivos</t>
   </si>
   <si>
-    <t>Derecho</t>
-  </si>
-  <si>
-    <t>Administración de Empresas</t>
-  </si>
-  <si>
-    <t>1053805543</t>
-  </si>
-  <si>
     <t>Elvia Lucía Sanchez García</t>
   </si>
   <si>
-    <t>Carlos Morales</t>
-  </si>
-  <si>
-    <t>sebas</t>
-  </si>
-  <si>
     <t>Juan Pablo Charry</t>
   </si>
   <si>
-    <t>María Eugenia Nieto</t>
+    <t>Temas_Centro_Escritura</t>
+  </si>
+  <si>
+    <t>Alfonso, Virtual</t>
+  </si>
+  <si>
+    <t>Cien años de soledad</t>
+  </si>
+  <si>
+    <t>Álvaro Agudelo</t>
   </si>
   <si>
     <t>Harold Estiven García</t>
   </si>
   <si>
-    <t>Temas_Centro_Escritura</t>
-  </si>
-  <si>
-    <t>APA _(7 ed. 2020)_American_Psychological_Association.</t>
-  </si>
-  <si>
-    <t>Alfonso, Virtual</t>
-  </si>
-  <si>
-    <t>Gonzalo Gallego, Presencial</t>
-  </si>
-  <si>
-    <t>Cien años de soledad</t>
-  </si>
-  <si>
-    <t>Prueba</t>
-  </si>
-  <si>
-    <t>Álvaro Agudelo</t>
-  </si>
-  <si>
     <t>ok</t>
   </si>
   <si>
     <t>Sí</t>
   </si>
   <si>
-    <t>No</t>
-  </si>
-  <si>
     <t>Presencial</t>
   </si>
   <si>
-    <t>Virtual</t>
-  </si>
-  <si>
     <t>Temas_Centro_Escritura | IEEE_(2025)_Institute_of_Electrical_and_Electronics_Engineers</t>
   </si>
   <si>
     <t>Juan Pablo Charry | Diego López, Presencial | Diego Alejandro Soto</t>
   </si>
   <si>
-    <t>2026-02-23</t>
-  </si>
-  <si>
-    <t>2026-02-22</t>
-  </si>
-  <si>
     <t>EN PROCESO</t>
-  </si>
-  <si>
-    <t>Si</t>
-  </si>
-  <si>
-    <t>En proceso</t>
   </si>
   <si>
     <t>alfonso</t>
@@ -555,7 +504,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AA4"/>
+  <dimension ref="A1:AA2"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:27">
@@ -646,197 +595,67 @@
         <v>27</v>
       </c>
       <c r="B2" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="C2">
         <v>1053766068</v>
       </c>
       <c r="D2" t="s">
-        <v>34</v>
+        <v>29</v>
       </c>
       <c r="E2" t="s">
-        <v>37</v>
+        <v>30</v>
       </c>
       <c r="F2" t="s">
-        <v>40</v>
+        <v>31</v>
       </c>
       <c r="H2" t="s">
-        <v>42</v>
+        <v>32</v>
       </c>
       <c r="I2" t="s">
-        <v>44</v>
+        <v>33</v>
       </c>
       <c r="J2" s="2">
         <v>46073</v>
       </c>
       <c r="K2" t="s">
-        <v>46</v>
+        <v>34</v>
       </c>
       <c r="L2" t="s">
-        <v>39</v>
+        <v>35</v>
       </c>
       <c r="N2" t="s">
-        <v>47</v>
+        <v>36</v>
       </c>
       <c r="P2" t="s">
-        <v>48</v>
+        <v>37</v>
       </c>
       <c r="Q2">
         <v>0</v>
       </c>
       <c r="R2" t="s">
-        <v>48</v>
+        <v>37</v>
       </c>
       <c r="S2" t="s">
-        <v>50</v>
+        <v>38</v>
       </c>
       <c r="T2">
         <v>2</v>
       </c>
       <c r="U2" t="s">
-        <v>52</v>
+        <v>39</v>
       </c>
       <c r="V2" t="s">
-        <v>53</v>
+        <v>40</v>
       </c>
       <c r="X2" t="s">
-        <v>56</v>
+        <v>41</v>
       </c>
       <c r="Z2" t="s">
-        <v>37</v>
+        <v>30</v>
       </c>
       <c r="AA2" t="s">
-        <v>59</v>
-      </c>
-    </row>
-    <row r="3" spans="1:27">
-      <c r="A3" t="s">
-        <v>28</v>
-      </c>
-      <c r="B3" t="s">
-        <v>31</v>
-      </c>
-      <c r="C3">
-        <v>123456</v>
-      </c>
-      <c r="D3" t="s">
-        <v>35</v>
-      </c>
-      <c r="E3" t="s">
-        <v>38</v>
-      </c>
-      <c r="F3" t="s">
-        <v>41</v>
-      </c>
-      <c r="H3" t="s">
-        <v>43</v>
-      </c>
-      <c r="I3" t="s">
-        <v>45</v>
-      </c>
-      <c r="J3" s="2">
-        <v>46076</v>
-      </c>
-      <c r="K3" t="s">
-        <v>46</v>
-      </c>
-      <c r="L3" t="s">
-        <v>39</v>
-      </c>
-      <c r="M3" t="s">
-        <v>47</v>
-      </c>
-      <c r="N3" t="s">
-        <v>47</v>
-      </c>
-      <c r="P3" t="s">
-        <v>48</v>
-      </c>
-      <c r="Q3">
-        <v>4</v>
-      </c>
-      <c r="R3" t="s">
-        <v>49</v>
-      </c>
-      <c r="S3" t="s">
-        <v>51</v>
-      </c>
-      <c r="T3">
-        <v>1</v>
-      </c>
-      <c r="U3" t="s">
-        <v>41</v>
-      </c>
-      <c r="W3" t="s">
-        <v>54</v>
-      </c>
-      <c r="X3" t="s">
-        <v>57</v>
-      </c>
-      <c r="Z3" t="s">
-        <v>38</v>
-      </c>
-      <c r="AA3" t="s">
-        <v>43</v>
-      </c>
-    </row>
-    <row r="4" spans="1:27">
-      <c r="A4" t="s">
-        <v>29</v>
-      </c>
-      <c r="B4" t="s">
-        <v>32</v>
-      </c>
-      <c r="C4" t="s">
-        <v>33</v>
-      </c>
-      <c r="D4" t="s">
-        <v>36</v>
-      </c>
-      <c r="E4" t="s">
-        <v>39</v>
-      </c>
-      <c r="F4" t="s">
-        <v>41</v>
-      </c>
-      <c r="I4" t="s">
-        <v>44</v>
-      </c>
-      <c r="J4" s="2">
-        <v>46075</v>
-      </c>
-      <c r="K4" t="s">
-        <v>46</v>
-      </c>
-      <c r="L4" t="s">
-        <v>39</v>
-      </c>
-      <c r="P4" t="s">
-        <v>48</v>
-      </c>
-      <c r="Q4">
-        <v>0</v>
-      </c>
-      <c r="R4" t="s">
-        <v>48</v>
-      </c>
-      <c r="S4" t="s">
-        <v>51</v>
-      </c>
-      <c r="T4">
-        <v>1</v>
-      </c>
-      <c r="U4" t="s">
-        <v>41</v>
-      </c>
-      <c r="W4" t="s">
-        <v>55</v>
-      </c>
-      <c r="X4" t="s">
-        <v>58</v>
-      </c>
-      <c r="Z4" t="s">
-        <v>39</v>
+        <v>42</v>
       </c>
     </row>
   </sheetData>

</xml_diff>